<commit_message>
added notes to .xlsx file
</commit_message>
<xml_diff>
--- a/BW-Dev/CharacterizeRunnables/RunnableFileResults.xlsx
+++ b/BW-Dev/CharacterizeRunnables/RunnableFileResults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brian/Documents/GitHub/Whirlwind-Instruction-Simulator/BW-Dev/CharacterizeRunnables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6B83D9F-7C81-EB4F-B8AE-3F4EFF499C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D9C72B91-172F-6B46-87C8-C7DF58216F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="55400" yWindow="1380" windowWidth="27640" windowHeight="16680" xr2:uid="{460DF726-D983-4341-A6E5-C63CC5C903FB}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="411">
   <si>
     <t>FileName</t>
   </si>
@@ -1172,6 +1172,87 @@
   </si>
   <si>
     <t>Halt Instruction!  (Code=0) at pc=01112</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Makes a big "X" on the screen</t>
+  </si>
+  <si>
+    <t>makes an array of little rectangles on screen</t>
+  </si>
+  <si>
+    <t>looks like it's trying to write 72 on the screen</t>
+  </si>
+  <si>
+    <t>draws array of "+" on screen</t>
+  </si>
+  <si>
+    <t>some sort of clickable game?</t>
+  </si>
+  <si>
+    <t>bouncing ball</t>
+  </si>
+  <si>
+    <t>plots what looks like a sine curve</t>
+  </si>
+  <si>
+    <t>tries to draw some #s on screen</t>
+  </si>
+  <si>
+    <t>draws some dots in upper right corner</t>
+  </si>
+  <si>
+    <t>could be Nim?</t>
+  </si>
+  <si>
+    <t>writes "FB125" and part of coordinate axes</t>
+  </si>
+  <si>
+    <t>nothing visible</t>
+  </si>
+  <si>
+    <t>prints "Amount of Sale:" - a change-making program?</t>
+  </si>
+  <si>
+    <t>looks like it's doing bulk transfers to flexo</t>
+  </si>
+  <si>
+    <t>prints "SELECT UNIT:" and halts</t>
+  </si>
+  <si>
+    <t>prints "Set core field switches to (2,0), then SA 40" then halts</t>
+  </si>
+  <si>
+    <t>prints '	0.00200	0.04000	0.02000"</t>
+  </si>
+  <si>
+    <t>prints "0.00200	0.14000	0.02001"</t>
+  </si>
+  <si>
+    <t>prints "0.00200	0.24040	0.00641"</t>
+  </si>
+  <si>
+    <t>prints "	0.00200	0.12000	0.02000"</t>
+  </si>
+  <si>
+    <t>prints "0.00200	0.30040	0.01741"</t>
+  </si>
+  <si>
+    <t>prints "	0.00200	0.44040	0.00540"</t>
+  </si>
+  <si>
+    <t>prints "0.00200	0.10000	0.02000"</t>
+  </si>
+  <si>
+    <t>prints "0.00200	0.06000	0.02000"</t>
+  </si>
+  <si>
+    <t>prints "	0.00200	0.22000	0.02000"</t>
+  </si>
+  <si>
+    <t>prints "PRINT 20 CHARACTERS FOR si230 CHECK"</t>
   </si>
 </sst>
 </file>
@@ -2032,10 +2113,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06B8FE15-5891-8D42-8CB3-3C0015EEB73A}">
-  <dimension ref="A1:I259"/>
+  <dimension ref="A1:J259"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="48.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="47.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2063,8 +2154,11 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J1" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -2093,7 +2187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -2122,7 +2216,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -2150,8 +2244,11 @@
       <c r="I4">
         <v>177.3</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J4" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2180,7 +2277,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -2209,7 +2306,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -2238,7 +2335,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -2267,7 +2364,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -2296,7 +2393,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -2325,7 +2422,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -2354,7 +2451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -2383,7 +2480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -2412,7 +2509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -2441,7 +2538,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2470,7 +2567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>34</v>
       </c>
@@ -2960,7 +3057,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>60</v>
       </c>
@@ -2989,7 +3086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>61</v>
       </c>
@@ -3018,7 +3115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>63</v>
       </c>
@@ -3047,7 +3144,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>65</v>
       </c>
@@ -3076,7 +3173,7 @@
         <v>45.8</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>67</v>
       </c>
@@ -3104,8 +3201,11 @@
       <c r="I37">
         <v>62.4</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J37" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>69</v>
       </c>
@@ -3134,7 +3234,7 @@
         <v>20.3</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>71</v>
       </c>
@@ -3163,7 +3263,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>72</v>
       </c>
@@ -3192,7 +3292,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>73</v>
       </c>
@@ -3221,7 +3321,7 @@
         <v>163.6</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>75</v>
       </c>
@@ -3250,7 +3350,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>76</v>
       </c>
@@ -3279,7 +3379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>78</v>
       </c>
@@ -3308,7 +3408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>80</v>
       </c>
@@ -3337,7 +3437,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>82</v>
       </c>
@@ -3366,7 +3466,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>83</v>
       </c>
@@ -3395,7 +3495,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>84</v>
       </c>
@@ -3424,7 +3524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>86</v>
       </c>
@@ -3452,8 +3552,11 @@
       <c r="I49">
         <v>6.6</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J49" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>88</v>
       </c>
@@ -3482,7 +3585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>89</v>
       </c>
@@ -3511,7 +3614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>90</v>
       </c>
@@ -3540,7 +3643,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>92</v>
       </c>
@@ -3569,7 +3672,7 @@
         <v>9.6999999999999993</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>94</v>
       </c>
@@ -3598,7 +3701,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>95</v>
       </c>
@@ -3627,7 +3730,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>96</v>
       </c>
@@ -3656,7 +3759,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>97</v>
       </c>
@@ -3685,7 +3788,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>99</v>
       </c>
@@ -3714,7 +3817,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>100</v>
       </c>
@@ -3743,7 +3846,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>101</v>
       </c>
@@ -3772,7 +3875,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>102</v>
       </c>
@@ -3801,7 +3904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>104</v>
       </c>
@@ -3829,8 +3932,11 @@
       <c r="I62">
         <v>553.70000000000005</v>
       </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J62" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>106</v>
       </c>
@@ -3859,7 +3965,7 @@
         <v>470.3</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>108</v>
       </c>
@@ -3888,7 +3994,7 @@
         <v>470.3</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>109</v>
       </c>
@@ -3917,7 +4023,7 @@
         <v>470.3</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>110</v>
       </c>
@@ -3946,7 +4052,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>112</v>
       </c>
@@ -3975,7 +4081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>114</v>
       </c>
@@ -4004,7 +4110,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>116</v>
       </c>
@@ -4033,7 +4139,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>118</v>
       </c>
@@ -4062,7 +4168,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>120</v>
       </c>
@@ -4091,7 +4197,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>122</v>
       </c>
@@ -4120,7 +4226,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>124</v>
       </c>
@@ -4149,7 +4255,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>125</v>
       </c>
@@ -4178,7 +4284,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>127</v>
       </c>
@@ -4206,8 +4312,11 @@
       <c r="I75">
         <v>49.5</v>
       </c>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J75" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>129</v>
       </c>
@@ -4236,7 +4345,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>131</v>
       </c>
@@ -4265,7 +4374,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>132</v>
       </c>
@@ -4294,7 +4403,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>133</v>
       </c>
@@ -4323,7 +4432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>135</v>
       </c>
@@ -4352,7 +4461,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>136</v>
       </c>
@@ -4381,7 +4490,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>138</v>
       </c>
@@ -4410,7 +4519,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>139</v>
       </c>
@@ -4439,7 +4548,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>140</v>
       </c>
@@ -4468,7 +4577,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>142</v>
       </c>
@@ -4497,7 +4606,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>144</v>
       </c>
@@ -4526,7 +4635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>145</v>
       </c>
@@ -4555,7 +4664,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>147</v>
       </c>
@@ -4584,7 +4693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>148</v>
       </c>
@@ -4613,7 +4722,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>149</v>
       </c>
@@ -4642,7 +4751,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>150</v>
       </c>
@@ -4671,7 +4780,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>151</v>
       </c>
@@ -4700,7 +4809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>152</v>
       </c>
@@ -4728,8 +4837,11 @@
       <c r="I93">
         <v>21</v>
       </c>
-    </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J93" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>154</v>
       </c>
@@ -4758,7 +4870,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>156</v>
       </c>
@@ -4787,7 +4899,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>157</v>
       </c>
@@ -4816,7 +4928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>158</v>
       </c>
@@ -4845,7 +4957,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>159</v>
       </c>
@@ -4874,7 +4986,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>161</v>
       </c>
@@ -4903,7 +5015,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>162</v>
       </c>
@@ -4932,7 +5044,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>163</v>
       </c>
@@ -4961,7 +5073,7 @@
         <v>8.3000000000000007</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>165</v>
       </c>
@@ -4990,7 +5102,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>166</v>
       </c>
@@ -5019,7 +5131,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>168</v>
       </c>
@@ -5048,7 +5160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>170</v>
       </c>
@@ -5077,7 +5189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>172</v>
       </c>
@@ -5106,7 +5218,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>173</v>
       </c>
@@ -5135,7 +5247,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>174</v>
       </c>
@@ -5164,7 +5276,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>176</v>
       </c>
@@ -5193,7 +5305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>177</v>
       </c>
@@ -5218,8 +5330,11 @@
       <c r="I110">
         <v>5.3</v>
       </c>
-    </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J110" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>178</v>
       </c>
@@ -5248,7 +5363,7 @@
         <v>42.7</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>180</v>
       </c>
@@ -5277,7 +5392,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>182</v>
       </c>
@@ -5306,7 +5421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>184</v>
       </c>
@@ -5335,7 +5450,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>185</v>
       </c>
@@ -5364,7 +5479,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>186</v>
       </c>
@@ -5393,7 +5508,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>187</v>
       </c>
@@ -5422,7 +5537,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>188</v>
       </c>
@@ -5451,7 +5566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>189</v>
       </c>
@@ -5480,7 +5595,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>190</v>
       </c>
@@ -5509,7 +5624,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>191</v>
       </c>
@@ -5538,7 +5653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>192</v>
       </c>
@@ -5567,7 +5682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>194</v>
       </c>
@@ -5596,7 +5711,7 @@
         <v>4999</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>196</v>
       </c>
@@ -5625,7 +5740,7 @@
         <v>499.8</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>198</v>
       </c>
@@ -5650,8 +5765,11 @@
       <c r="I125">
         <v>7.8</v>
       </c>
-    </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J125" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>199</v>
       </c>
@@ -5680,7 +5798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>201</v>
       </c>
@@ -5709,7 +5827,7 @@
         <v>70.400000000000006</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>203</v>
       </c>
@@ -5738,7 +5856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>204</v>
       </c>
@@ -5767,7 +5885,7 @@
         <v>470.3</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>205</v>
       </c>
@@ -5796,7 +5914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>206</v>
       </c>
@@ -5825,7 +5943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>208</v>
       </c>
@@ -5854,7 +5972,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>209</v>
       </c>
@@ -5883,7 +6001,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>210</v>
       </c>
@@ -5912,7 +6030,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>211</v>
       </c>
@@ -5941,7 +6059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>213</v>
       </c>
@@ -5970,7 +6088,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>215</v>
       </c>
@@ -5999,7 +6117,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>216</v>
       </c>
@@ -6028,7 +6146,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>217</v>
       </c>
@@ -6057,7 +6175,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>218</v>
       </c>
@@ -6086,7 +6204,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>220</v>
       </c>
@@ -6112,7 +6230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>221</v>
       </c>
@@ -6141,7 +6259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>223</v>
       </c>
@@ -6169,8 +6287,11 @@
       <c r="I143">
         <v>42</v>
       </c>
-    </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J143" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>225</v>
       </c>
@@ -6199,7 +6320,7 @@
         <v>135.6</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>227</v>
       </c>
@@ -6228,7 +6349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>228</v>
       </c>
@@ -6257,7 +6378,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>229</v>
       </c>
@@ -6286,7 +6407,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>230</v>
       </c>
@@ -6315,7 +6436,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>232</v>
       </c>
@@ -6344,7 +6465,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>234</v>
       </c>
@@ -6372,8 +6493,11 @@
       <c r="I150">
         <v>212.9</v>
       </c>
-    </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J150" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>236</v>
       </c>
@@ -6402,7 +6526,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>238</v>
       </c>
@@ -6431,7 +6555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>240</v>
       </c>
@@ -6460,7 +6584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>242</v>
       </c>
@@ -6489,7 +6613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>244</v>
       </c>
@@ -6517,8 +6641,11 @@
       <c r="I155">
         <v>138.1</v>
       </c>
-    </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J155" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>246</v>
       </c>
@@ -6547,7 +6674,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>247</v>
       </c>
@@ -6576,7 +6703,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>248</v>
       </c>
@@ -6605,7 +6732,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>249</v>
       </c>
@@ -6634,7 +6761,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>250</v>
       </c>
@@ -6663,7 +6790,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>251</v>
       </c>
@@ -6692,7 +6819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>252</v>
       </c>
@@ -6721,7 +6848,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>253</v>
       </c>
@@ -6750,7 +6877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>255</v>
       </c>
@@ -6779,7 +6906,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>256</v>
       </c>
@@ -6808,7 +6935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>258</v>
       </c>
@@ -6837,7 +6964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>259</v>
       </c>
@@ -6866,7 +6993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>261</v>
       </c>
@@ -6895,7 +7022,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>263</v>
       </c>
@@ -6924,7 +7051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>264</v>
       </c>
@@ -6952,8 +7079,11 @@
       <c r="I170">
         <v>7</v>
       </c>
-    </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J170" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>266</v>
       </c>
@@ -6978,8 +7108,11 @@
       <c r="I171">
         <v>5</v>
       </c>
-    </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J171" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="172" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>267</v>
       </c>
@@ -7008,7 +7141,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>268</v>
       </c>
@@ -7037,7 +7170,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>269</v>
       </c>
@@ -7066,7 +7199,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>271</v>
       </c>
@@ -7095,7 +7228,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>273</v>
       </c>
@@ -7120,8 +7253,11 @@
       <c r="I176">
         <v>5</v>
       </c>
-    </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J176" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="177" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>274</v>
       </c>
@@ -7150,7 +7286,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>275</v>
       </c>
@@ -7175,8 +7311,11 @@
       <c r="I178">
         <v>5</v>
       </c>
-    </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J178" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="179" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>276</v>
       </c>
@@ -7205,7 +7344,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>277</v>
       </c>
@@ -7234,7 +7373,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>278</v>
       </c>
@@ -7263,7 +7402,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>279</v>
       </c>
@@ -7288,8 +7427,11 @@
       <c r="I182">
         <v>5</v>
       </c>
-    </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J182" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="183" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>280</v>
       </c>
@@ -7318,7 +7460,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>281</v>
       </c>
@@ -7343,8 +7485,11 @@
       <c r="I184">
         <v>5</v>
       </c>
-    </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J184" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="185" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>282</v>
       </c>
@@ -7373,7 +7518,7 @@
         <v>203.4</v>
       </c>
     </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>283</v>
       </c>
@@ -7398,8 +7543,11 @@
       <c r="I186">
         <v>5</v>
       </c>
-    </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J186" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="187" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>284</v>
       </c>
@@ -7428,7 +7576,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>285</v>
       </c>
@@ -7457,7 +7605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>287</v>
       </c>
@@ -7486,7 +7634,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>288</v>
       </c>
@@ -7511,8 +7659,11 @@
       <c r="I190">
         <v>5</v>
       </c>
-    </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J190" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="191" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>289</v>
       </c>
@@ -7541,7 +7692,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>290</v>
       </c>
@@ -7570,7 +7721,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>291</v>
       </c>
@@ -7599,7 +7750,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>292</v>
       </c>
@@ -7628,7 +7779,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>293</v>
       </c>
@@ -7657,7 +7808,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>294</v>
       </c>
@@ -7682,8 +7833,11 @@
       <c r="I196">
         <v>5</v>
       </c>
-    </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J196" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="197" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>295</v>
       </c>
@@ -7712,7 +7866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>296</v>
       </c>
@@ -7741,7 +7895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>297</v>
       </c>
@@ -7770,7 +7924,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>298</v>
       </c>
@@ -7799,7 +7953,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>300</v>
       </c>
@@ -7827,8 +7981,11 @@
       <c r="I201">
         <v>52</v>
       </c>
-    </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J201" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="202" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>302</v>
       </c>
@@ -7857,7 +8014,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>303</v>
       </c>
@@ -7886,7 +8043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>305</v>
       </c>
@@ -7915,7 +8072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>307</v>
       </c>
@@ -7944,7 +8101,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>309</v>
       </c>
@@ -7973,7 +8130,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>310</v>
       </c>
@@ -8002,7 +8159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>311</v>
       </c>
@@ -8031,7 +8188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>313</v>
       </c>
@@ -8060,7 +8217,7 @@
         <v>2500</v>
       </c>
     </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>315</v>
       </c>
@@ -8089,7 +8246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>316</v>
       </c>
@@ -8118,7 +8275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>317</v>
       </c>
@@ -8147,7 +8304,7 @@
         <v>470.3</v>
       </c>
     </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>318</v>
       </c>
@@ -8176,7 +8333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>319</v>
       </c>
@@ -8205,7 +8362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>320</v>
       </c>
@@ -8234,7 +8391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>321</v>
       </c>
@@ -8263,7 +8420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>322</v>
       </c>
@@ -8292,7 +8449,7 @@
         <v>470.3</v>
       </c>
     </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>323</v>
       </c>
@@ -8320,8 +8477,11 @@
       <c r="I218">
         <v>61.5</v>
       </c>
-    </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J218" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="219" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>325</v>
       </c>
@@ -8350,7 +8510,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>326</v>
       </c>
@@ -8379,7 +8539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>327</v>
       </c>
@@ -8408,7 +8568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>329</v>
       </c>
@@ -8433,8 +8593,11 @@
       <c r="I222">
         <v>15.7</v>
       </c>
-    </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J222" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="223" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>330</v>
       </c>
@@ -8462,8 +8625,11 @@
       <c r="I223">
         <v>34.6</v>
       </c>
-    </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J223" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="224" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>332</v>
       </c>
@@ -8491,8 +8657,11 @@
       <c r="I224">
         <v>28.6</v>
       </c>
-    </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J224" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="225" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>334</v>
       </c>
@@ -8521,7 +8690,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>336</v>
       </c>
@@ -8549,8 +8718,11 @@
       <c r="I226">
         <v>1</v>
       </c>
-    </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J226" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="227" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>338</v>
       </c>
@@ -8579,7 +8751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>339</v>
       </c>
@@ -8608,7 +8780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>340</v>
       </c>
@@ -8637,7 +8809,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>341</v>
       </c>
@@ -8666,7 +8838,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>342</v>
       </c>
@@ -8695,7 +8867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>344</v>
       </c>
@@ -8724,7 +8896,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>345</v>
       </c>
@@ -8753,7 +8925,7 @@
         <v>20.3</v>
       </c>
     </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>346</v>
       </c>
@@ -8782,7 +8954,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>348</v>
       </c>
@@ -8810,8 +8982,11 @@
       <c r="I235">
         <v>62.4</v>
       </c>
-    </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J235" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="236" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>349</v>
       </c>
@@ -8840,7 +9015,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>351</v>
       </c>
@@ -8869,7 +9044,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>353</v>
       </c>
@@ -8898,7 +9073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>354</v>
       </c>
@@ -8927,7 +9102,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>355</v>
       </c>

</xml_diff>

<commit_message>
more details in xlsx
</commit_message>
<xml_diff>
--- a/BW-Dev/CharacterizeRunnables/RunnableFileResults.xlsx
+++ b/BW-Dev/CharacterizeRunnables/RunnableFileResults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brian/Documents/GitHub/Whirlwind-Instruction-Simulator/BW-Dev/CharacterizeRunnables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{E20836D9-6FA8-A24A-9547-8C128A9AAD42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{07E3D89C-986A-534E-B24C-83922CC79735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="55400" yWindow="1380" windowWidth="27640" windowHeight="16680" xr2:uid="{460DF726-D983-4341-A6E5-C63CC5C903FB}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="412">
   <si>
     <t>FileName</t>
   </si>
@@ -1207,9 +1207,6 @@
     <t>writes "FB125" and part of coordinate axes</t>
   </si>
   <si>
-    <t>nothing visible</t>
-  </si>
-  <si>
     <t>prints "Amount of Sale:" - a change-making program?</t>
   </si>
   <si>
@@ -1253,6 +1250,12 @@
   </si>
   <si>
     <t>this is NIM</t>
+  </si>
+  <si>
+    <t>blackjack?</t>
+  </si>
+  <si>
+    <t>nothing visible - blackjack?</t>
   </si>
 </sst>
 </file>
@@ -3933,7 +3936,7 @@
         <v>553.70000000000005</v>
       </c>
       <c r="J62" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
@@ -4313,7 +4316,7 @@
         <v>49.5</v>
       </c>
       <c r="J75" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.2">
@@ -5331,7 +5334,7 @@
         <v>5.3</v>
       </c>
       <c r="J110" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.2">
@@ -5766,7 +5769,7 @@
         <v>7.8</v>
       </c>
       <c r="J125" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.2">
@@ -7080,7 +7083,7 @@
         <v>7</v>
       </c>
       <c r="J170" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="171" spans="1:10" x14ac:dyDescent="0.2">
@@ -7109,7 +7112,7 @@
         <v>5</v>
       </c>
       <c r="J171" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="172" spans="1:10" x14ac:dyDescent="0.2">
@@ -7254,7 +7257,7 @@
         <v>5</v>
       </c>
       <c r="J176" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="177" spans="1:10" x14ac:dyDescent="0.2">
@@ -7312,7 +7315,7 @@
         <v>5</v>
       </c>
       <c r="J178" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="179" spans="1:10" x14ac:dyDescent="0.2">
@@ -7428,7 +7431,7 @@
         <v>5</v>
       </c>
       <c r="J182" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="183" spans="1:10" x14ac:dyDescent="0.2">
@@ -7486,7 +7489,7 @@
         <v>5</v>
       </c>
       <c r="J184" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="185" spans="1:10" x14ac:dyDescent="0.2">
@@ -7544,7 +7547,7 @@
         <v>5</v>
       </c>
       <c r="J186" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.2">
@@ -7660,7 +7663,7 @@
         <v>5</v>
       </c>
       <c r="J190" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="191" spans="1:10" x14ac:dyDescent="0.2">
@@ -7834,7 +7837,7 @@
         <v>5</v>
       </c>
       <c r="J196" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="197" spans="1:10" x14ac:dyDescent="0.2">
@@ -8594,7 +8597,7 @@
         <v>15.7</v>
       </c>
       <c r="J222" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="223" spans="1:10" x14ac:dyDescent="0.2">
@@ -8626,7 +8629,7 @@
         <v>34.6</v>
       </c>
       <c r="J223" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="224" spans="1:10" x14ac:dyDescent="0.2">
@@ -8689,6 +8692,9 @@
       <c r="I225" t="s">
         <v>13</v>
       </c>
+      <c r="J225" t="s">
+        <v>410</v>
+      </c>
     </row>
     <row r="226" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
@@ -8719,7 +8725,7 @@
         <v>1</v>
       </c>
       <c r="J226" t="s">
-        <v>395</v>
+        <v>411</v>
       </c>
     </row>
     <row r="227" spans="1:10" x14ac:dyDescent="0.2">

</xml_diff>